<commit_message>
feat: onconformity relationship with photos
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luiz.defreitas\projects\gerador-de-relatorios\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{178D60EC-1A5A-49AD-BCEC-9C30A31F9D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C3BF0DC-6A5F-442A-A7BD-9BCE523BA633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="44">
   <si>
     <t>ID da Fiscalização</t>
   </si>
@@ -53,18 +53,9 @@
     <t>Observações</t>
   </si>
   <si>
-    <t>Fotos</t>
-  </si>
-  <si>
-    <t>Não conformidade</t>
-  </si>
-  <si>
     <t>Relatório Gerado</t>
   </si>
   <si>
-    <t>CTR 06/2031</t>
-  </si>
-  <si>
     <t>10:00:06</t>
   </si>
   <si>
@@ -89,16 +80,6 @@
     <t xml:space="preserve">Aqui vai as observaçoes da fiscalização </t>
   </si>
   <si>
-    <t>foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg</t>
-  </si>
-  <si>
-    <t>CIMENTO NÃO POSICIONADO 
-DE ACORDO COM ORIENTAÇÃO</t>
-  </si>
-  <si>
-    <t>CTR 06/2032</t>
-  </si>
-  <si>
     <t>10:00:07</t>
   </si>
   <si>
@@ -108,9 +89,6 @@
     <t>26/04/2025 a 01/05/2032</t>
   </si>
   <si>
-    <t>CTR 06/2033</t>
-  </si>
-  <si>
     <t>10:00:08</t>
   </si>
   <si>
@@ -120,9 +98,6 @@
     <t>26/04/2025 a 01/05/2033</t>
   </si>
   <si>
-    <t>CTR 06/2034</t>
-  </si>
-  <si>
     <t>10:00:09</t>
   </si>
   <si>
@@ -132,9 +107,6 @@
     <t>26/04/2025 a 01/05/2034</t>
   </si>
   <si>
-    <t>CTR 06/2035</t>
-  </si>
-  <si>
     <t>10:00:10</t>
   </si>
   <si>
@@ -144,9 +116,6 @@
     <t>26/04/2025 a 01/05/2035</t>
   </si>
   <si>
-    <t>CTR 06/2036</t>
-  </si>
-  <si>
     <t>10:00:11</t>
   </si>
   <si>
@@ -156,19 +125,34 @@
     <t>26/04/2025 a 01/05/2036</t>
   </si>
   <si>
-    <t>foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg;foto01.jpg;foto02.jpg</t>
+    <t>10:00:12</t>
+  </si>
+  <si>
+    <t>Nº 1.041.080/20</t>
+  </si>
+  <si>
+    <t>26/04/2025 a 01/05/2037</t>
   </si>
   <si>
     <t>Nº</t>
   </si>
   <si>
+    <t>Não Conformidade</t>
+  </si>
+  <si>
+    <t>Foto</t>
+  </si>
+  <si>
     <t>Legenda da Foto</t>
   </si>
   <si>
-    <t>Foto</t>
-  </si>
-  <si>
-    <t>Não Conformidade</t>
+    <t>CIMENTO NÃO POSICIONADO NA SACADA</t>
+  </si>
+  <si>
+    <t>foto01.jpg</t>
+  </si>
+  <si>
+    <t>Infiltração em coluna de sustentação do Terminal do recife</t>
   </si>
 </sst>
 </file>
@@ -535,7 +519,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -548,12 +532,10 @@
     <col min="8" max="8" width="17" customWidth="1"/>
     <col min="9" max="9" width="25" customWidth="1"/>
     <col min="10" max="10" width="42" customWidth="1"/>
-    <col min="11" max="11" width="793" customWidth="1"/>
-    <col min="12" max="12" width="51" customWidth="1"/>
-    <col min="13" max="13" width="18" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -587,256 +569,249 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>13</v>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2" s="2">
         <v>45816</v>
       </c>
       <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>16</v>
       </c>
-      <c r="F2" t="s">
+      <c r="I2" t="s">
         <v>17</v>
       </c>
-      <c r="G2" t="s">
+      <c r="J2" t="s">
         <v>18</v>
       </c>
-      <c r="H2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>24</v>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
       </c>
       <c r="B3" s="2">
         <v>45817</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" t="s">
         <v>18</v>
       </c>
-      <c r="H3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K3" t="s">
-        <v>22</v>
-      </c>
-      <c r="L3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>28</v>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
       </c>
       <c r="B4" s="2">
         <v>45818</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
         <v>15</v>
       </c>
-      <c r="E4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" t="s">
         <v>18</v>
       </c>
-      <c r="H4" t="s">
-        <v>30</v>
-      </c>
-      <c r="I4" t="s">
-        <v>31</v>
-      </c>
-      <c r="J4" t="s">
-        <v>21</v>
-      </c>
-      <c r="K4" t="s">
-        <v>22</v>
-      </c>
-      <c r="L4" t="s">
-        <v>23</v>
-      </c>
-      <c r="M4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>32</v>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
       </c>
       <c r="B5" s="2">
         <v>45819</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
         <v>15</v>
       </c>
-      <c r="E5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" t="s">
         <v>18</v>
       </c>
-      <c r="H5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I5" t="s">
-        <v>35</v>
-      </c>
-      <c r="J5" t="s">
-        <v>21</v>
-      </c>
-      <c r="K5" t="s">
-        <v>22</v>
-      </c>
-      <c r="L5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>36</v>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
       </c>
       <c r="B6" s="2">
         <v>45820</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
         <v>15</v>
       </c>
-      <c r="E6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" t="s">
+        <v>30</v>
+      </c>
+      <c r="J6" t="s">
         <v>18</v>
       </c>
-      <c r="H6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I6" t="s">
-        <v>39</v>
-      </c>
-      <c r="J6" t="s">
-        <v>21</v>
-      </c>
-      <c r="K6" t="s">
-        <v>22</v>
-      </c>
-      <c r="L6" t="s">
-        <v>23</v>
-      </c>
-      <c r="M6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>40</v>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
       </c>
       <c r="B7" s="2">
         <v>45821</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
         <v>15</v>
       </c>
-      <c r="E7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J7" t="s">
         <v>18</v>
       </c>
-      <c r="H7" t="s">
-        <v>42</v>
-      </c>
-      <c r="I7" t="s">
-        <v>43</v>
-      </c>
-      <c r="J7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K7" t="s">
-        <v>44</v>
-      </c>
-      <c r="L7" t="s">
-        <v>23</v>
-      </c>
-      <c r="M7" t="b">
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <v>45822</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I8" t="s">
+        <v>36</v>
+      </c>
+      <c r="J8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -846,35 +821,300 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D731C6E-F15F-4310-802E-7A32E5DFEE61}">
-  <dimension ref="A1:E1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="29.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.42578125" customWidth="1"/>
-    <col min="5" max="5" width="33.140625" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>1.2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>1.3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>1.4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>1.5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7">
+        <v>1.6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>1.7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9">
+        <v>1.8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>7</v>
+      </c>
+      <c r="B10">
+        <v>7.1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11">
+        <v>7.2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>7</v>
+      </c>
+      <c r="B12">
+        <v>7.3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>7</v>
+      </c>
+      <c r="B13">
+        <v>7.4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>7</v>
+      </c>
+      <c r="B14">
+        <v>7.5</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>7</v>
+      </c>
+      <c r="B15">
+        <v>7.6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>7</v>
+      </c>
+      <c r="B16">
+        <v>7.7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>7</v>
+      </c>
+      <c r="B17">
+        <v>7.8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: formatting date field
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -9,6 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscalizações" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Não-conformidades " sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observações Importantes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recomendações" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -17,10 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -31,11 +29,13 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -110,15 +110,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -488,7 +489,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="37" customWidth="1" min="5" max="5"/>
@@ -501,57 +502,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Cidade</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Pessoal Responsável</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Coordenador</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Contrato</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Período</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Assinatura</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>Relatório Gerado</t>
         </is>
@@ -561,8 +562,10 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="n">
-        <v>45816</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>08/06/2025</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -612,8 +615,10 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="n">
-        <v>45817</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>09/06/2025</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -663,8 +668,10 @@
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="8" t="n">
-        <v>45818</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10/06/2025</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -714,8 +721,10 @@
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="n">
-        <v>45819</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>11/06/2025</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -765,8 +774,10 @@
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="n">
-        <v>45820</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>12/06/2025</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -816,8 +827,10 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="n">
-        <v>45821</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>13/06/2025</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -867,8 +880,10 @@
       <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="8" t="n">
-        <v>45822</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>14/06/2025</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -918,8 +933,10 @@
       <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="8" t="n">
-        <v>45823</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>15/06/2025</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -969,8 +986,10 @@
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="8" t="n">
-        <v>45824</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>16/06/2025</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1020,8 +1039,10 @@
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="n">
-        <v>45825</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>17/06/2025</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1071,8 +1092,10 @@
       <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="8" t="n">
-        <v>45826</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>18/06/2025</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1122,8 +1145,10 @@
       <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="8" t="n">
-        <v>45860</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>22/07/2025</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1184,32 +1209,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Nº</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Não Conformidade</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Foto</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Legenda da Foto</t>
         </is>
@@ -3117,102 +3142,95 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
-  <cols>
-    <col width="15.453125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="29.453125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="195.1796875" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="19.81640625" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="111.54296875" bestFit="1" customWidth="1" min="5" max="5"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>ID da Fiscalização</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Observações</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Foto</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Legenda da Foto</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="116.15" customFormat="1" customHeight="1" s="2">
-      <c r="A2" s="2" t="n">
+    <row r="2">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Lorem ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum.</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>foto01.jpg</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Viga do terminal não posicionada corretamente.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="43.5" customFormat="1" customHeight="1" s="3">
-      <c r="A3" s="3" t="n">
+    <row r="3">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Terminal de Caruaru</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Lorem ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum ipsum lorem pisum.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customFormat="1" customHeight="1" s="3">
-      <c r="A4" s="3" t="n">
+    <row r="4">
+      <c r="A4" t="n">
         <v>11</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>foto01.jpg</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>foto01.jpg</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Viga do terminal não posicionada corretamente.</t>
         </is>
@@ -3288,11 +3306,11 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="14" customHeight="1">
+    <row r="9">
       <c r="A9" t="n">
         <v>12</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Terminal do Recife (TIP)</t>
         </is>
@@ -3303,7 +3321,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="14" customHeight="1">
+    <row r="10">
       <c r="A10" t="n">
         <v>12</v>
       </c>
@@ -3359,6 +3377,87 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>ID da Fiscalização</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Recomendação</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Legenda da Foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Terminal de Garanhuns (GAR)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Viga do terminal não posicionada corretamente.;Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025.;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Terminal de Arcoverde (ARC)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Implementa validação de entrada, adiciona novos módulos e refatora a estrutura do gerador de relatórios
</commit_message>
<xml_diff>
--- a/src/planilha_fiscalizacao.xlsx
+++ b/src/planilha_fiscalizacao.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscalizações" sheetId="1" state="visible" r:id="rId1"/>
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -529,7 +529,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>08/06/2025</t>
+          <t>06/08/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>09/06/2025</t>
+          <t>06/09/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10/06/2025</t>
+          <t>06/10/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11/06/2025</t>
+          <t>06/11/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>12/06/2025</t>
+          <t>06/12/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1156,6 +1156,160 @@
         </is>
       </c>
       <c r="K13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06/12/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>10:00:18</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Recife</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Terminal Rodoviário do Recife - TIP</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Débora Marcolino e Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Maria Ângela Albuquerque de Freitas</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Nº 1.041.080/09</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>26/04/2025 a 01/05/2042</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Débora Marcolino;Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="K14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06/12/2027</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>10:00:19</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Recife</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Terminal Rodoviário do Recife - TIP</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Débora Marcolino e Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Maria Ângela Albuquerque de Freitas</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Nº 1.041.080/10</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>26/04/2025 a 01/05/2043</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Débora Marcolino;Enildo Manoel</t>
+        </is>
+      </c>
+      <c r="K15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>16</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Recife</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Terminal Rodoviário do Recife - TIP</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Thays Barbosa</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Maria Ângela Albuquerque de Freitas</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Nº 1.100.100/00</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>26/04/2025 a 01/05/2043</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Thays Barbosa</t>
+        </is>
+      </c>
+      <c r="K16" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1170,8 +1324,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:M93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="179" customWidth="1" min="4" max="4"/>
+    <col width="67" customWidth="1" min="5" max="5"/>
+    <col width="241" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="49" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
@@ -1204,6 +1373,41 @@
           <t>Legenda da Foto</t>
         </is>
       </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>ID da não conformidade</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Informação SOCICAM</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Constatação</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Análise da Arpe</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Informação SOCICAM carta</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Vistoria da Arpe</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Situação</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1232,6 +1436,26 @@
           <t>Infiltração em coluna de sustentação do Terminal do recife</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>3.4- CTR 02/2024</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A SOCICAM </t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conforme fiscalização realizada dia 25/09/2025 </t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>A Não Conformidade sanada.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -3092,6 +3316,747 @@
       <c r="F71" t="inlineStr">
         <is>
           <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>13</v>
+      </c>
+      <c r="B72" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>13</v>
+      </c>
+      <c r="B73" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Terminal de Arcoverde (ARC)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>13</v>
+      </c>
+      <c r="B74" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Terminal de Serra Talhada (SER)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>13</v>
+      </c>
+      <c r="B75" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Terminal do Recife (TIP)</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>13</v>
+      </c>
+      <c r="B76" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Terminal de Garanhuns (GAR)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>13</v>
+      </c>
+      <c r="B77" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>13</v>
+      </c>
+      <c r="B78" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>14</v>
+      </c>
+      <c r="B79" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>14</v>
+      </c>
+      <c r="B80" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Terminal de Garanhuns (GAR)</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>14</v>
+      </c>
+      <c r="B81" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Terminal de Serra Talhada (SER)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>14</v>
+      </c>
+      <c r="B82" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Terminal de Arcoverde (ARC)</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>14</v>
+      </c>
+      <c r="B83" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Terminal de Arcoverde (ARC)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>14</v>
+      </c>
+      <c r="B84" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Terminal do Recife (TIP)</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>14</v>
+      </c>
+      <c r="B85" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>14</v>
+      </c>
+      <c r="B86" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>14</v>
+      </c>
+      <c r="B87" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>14</v>
+      </c>
+      <c r="B88" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>15</v>
+      </c>
+      <c r="B89" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>3.4- CTR 02/2024</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A SOCICAM </t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conforme fiscalização realizada dia 25/09/2025 </t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>A Não Conformidade sanada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>15</v>
+      </c>
+      <c r="B90" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>3.4- CTR 02/2024</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A SOCICAM </t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conforme fiscalização realizada dia 25/09/2025 </t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>A Não Conformidade sanada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>15</v>
+      </c>
+      <c r="B91" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Terminal de Serra Talhada (SER)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Piso desgastado conforme evidência da foto 04.;Segunda legenda qualquer coisa. </t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>3.4- CTR 02/2024</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A SOCICAM </t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conforme fiscalização realizada dia 25/09/2025 </t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>A Não Conformidade sanada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>16</v>
+      </c>
+      <c r="B92" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Terminal de Serra Talhada (SER)</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Piso desgastado conforme evidência da foto 04.;Piso normal;</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>3.4- CTR 02/2024</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A SOCICAM </t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conforme fiscalização realizada dia 25/09/2025 </t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>A Não Conformidade sanada.</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Lorem Ipsum</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Lorem Ipsum</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>Lorem Ipsum</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>16</v>
+      </c>
+      <c r="B93" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Piso desgastado na entrada do banheiro feminino de CAR em 20/03/2025;</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Piso desgastado conforme evidência da foto 04.;Piso normal;</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>3.5- CTR 02/2024</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A SOCICAM </t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conforme fiscalização realizada dia 25/09/2025 </t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>A Não Conformidade sanada.</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Lorem Ipsum</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Lorem Ipsum</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>Lorem Ipsum</t>
         </is>
       </c>
     </row>
@@ -3106,8 +4071,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="596" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="171" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
@@ -3373,6 +4345,56 @@
       <c r="E13" t="inlineStr">
         <is>
           <t>Viga do terminal não posicionada corretamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>15</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Terminal de Caruaru (CAR)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.;Tambem foi observada a presenca de caracteres incompativeis com a resolucao de numero 198392, uma vez que o dispositivo de regulamentacao exige acompanhamento especial durante todo o ciclo; Observa-se tambem lorem ipsumlorem ipsum lorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsum.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>foto01.jpg</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Viga do terminal não posicionada corretamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Terminal de Garanhuns (GAR)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.;Tambem foi observada a presenca de caracteres incompativeis com a resolucao de numero 198392, uma vez que o dispositivo de regulamentacao exige acompanhamento especial durante todo o ciclo; Observa-se tambem lorem ipsumlorem ipsum lorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsum.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg;foto002.jpg</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Viga do terminal não posicionada corretamente.;Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025.;Não conformidade detectada conforme resolucao 12394.</t>
         </is>
       </c>
     </row>
@@ -3387,8 +4409,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="596" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="296" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
@@ -3477,6 +4506,31 @@
         </is>
       </c>
       <c r="E4" t="inlineStr">
+        <is>
+          <t>Viga do terminal não posicionada corretamente.;Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025.;Lorem ipsum Lorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsum</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Terminal do Recife (TIP)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Durante a fiscalização, foi observada a presença de cidadãos que ficaram fiscalizando o serviço conforme o andamento do mesmo. Precisamos mobilizar uma equipe que fiscalize os agentes e os cidadãos em campo.;Tambem foi observada a presenca de caracteres incompativeis com a resolucao de numero 198392, uma vez que o dispositivo de regulamentacao exige acompanhamento especial durante todo o ciclo; Observa-se tambem lorem ipsumlorem ipsum lorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsumlorem ipsum.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>foto01.jpg;foto02.jpg;foto01.jpg</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Viga do terminal não posicionada corretamente.;Piso desgastado na entrada do banheiro feminino do TIP em 20/03/2025.;Lorem ipsum Lorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsumLorem ipsum</t>
         </is>

</xml_diff>